<commit_message>
Add the Fit-Gap workbooks to the Document Register
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Common/BIBS_Register_BRD-00_Document_Register_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Common/BIBS_Register_BRD-00_Document_Register_v1.0.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'README'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Register'!$A$4:$J$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Register'!$A$4:$J$80</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Register'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Lists'!$1:$1</definedName>
   </definedNames>
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="D21" s="14" t="n">
-        <v>65</v>
+        <v>76</v>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
@@ -1053,7 +1053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4526,18 +4526,590 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" s="12" t="inlineStr">
+        <is>
+          <t>BRD-00</t>
+        </is>
+      </c>
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t>FitGap</t>
+        </is>
+      </c>
+      <c r="C70" s="12" t="inlineStr">
+        <is>
+          <t>Core Replacement BRD vs OOTB vs Best Practice</t>
+        </is>
+      </c>
+      <c r="D70" s="12" t="inlineStr">
+        <is>
+          <t>BIBS_FitGap_BRD-00_Core_Replacement_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+        </is>
+      </c>
+      <c r="E70" s="12" t="inlineStr">
+        <is>
+          <t>XLSX</t>
+        </is>
+      </c>
+      <c r="F70" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G70" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H70" s="12" t="inlineStr">
+        <is>
+          <t>BIBS Product Owner</t>
+        </is>
+      </c>
+      <c r="I70" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="J70" s="22" t="inlineStr">
+        <is>
+          <t>Issued for BDOI review</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="12" t="inlineStr">
+        <is>
+          <t>BRD-00</t>
+        </is>
+      </c>
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t>FitGap</t>
+        </is>
+      </c>
+      <c r="C71" s="12" t="inlineStr">
+        <is>
+          <t>Summary All BRDs</t>
+        </is>
+      </c>
+      <c r="D71" s="12" t="inlineStr">
+        <is>
+          <t>BIBS_FitGap_BRD-00_Summary_All_BRDs_v1.0</t>
+        </is>
+      </c>
+      <c r="E71" s="12" t="inlineStr">
+        <is>
+          <t>XLSX</t>
+        </is>
+      </c>
+      <c r="F71" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G71" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H71" s="12" t="inlineStr">
+        <is>
+          <t>BIBS Product Owner</t>
+        </is>
+      </c>
+      <c r="I71" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="J71" s="22" t="inlineStr">
+        <is>
+          <t>Issued for BDOI review</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="12" t="inlineStr">
+        <is>
+          <t>BRD-01</t>
+        </is>
+      </c>
+      <c r="B72" s="12" t="inlineStr">
+        <is>
+          <t>FitGap</t>
+        </is>
+      </c>
+      <c r="C72" s="12" t="inlineStr">
+        <is>
+          <t>New Business BRD vs OOTB vs Best Practice</t>
+        </is>
+      </c>
+      <c r="D72" s="12" t="inlineStr">
+        <is>
+          <t>BIBS_FitGap_BRD-01_New_Business_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+        </is>
+      </c>
+      <c r="E72" s="12" t="inlineStr">
+        <is>
+          <t>XLSX</t>
+        </is>
+      </c>
+      <c r="F72" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G72" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H72" s="12" t="inlineStr">
+        <is>
+          <t>BIBS Product Owner</t>
+        </is>
+      </c>
+      <c r="I72" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="J72" s="22" t="inlineStr">
+        <is>
+          <t>Issued for BDOI review</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="12" t="inlineStr">
+        <is>
+          <t>BRD-04</t>
+        </is>
+      </c>
+      <c r="B73" s="12" t="inlineStr">
+        <is>
+          <t>FitGap</t>
+        </is>
+      </c>
+      <c r="C73" s="12" t="inlineStr">
+        <is>
+          <t>Collections BRD vs OOTB vs Best Practice</t>
+        </is>
+      </c>
+      <c r="D73" s="12" t="inlineStr">
+        <is>
+          <t>BIBS_FitGap_BRD-04_Collections_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+        </is>
+      </c>
+      <c r="E73" s="12" t="inlineStr">
+        <is>
+          <t>XLSX</t>
+        </is>
+      </c>
+      <c r="F73" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G73" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H73" s="12" t="inlineStr">
+        <is>
+          <t>BIBS Product Owner</t>
+        </is>
+      </c>
+      <c r="I73" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="J73" s="22" t="inlineStr">
+        <is>
+          <t>Issued for BDOI review</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="12" t="inlineStr">
+        <is>
+          <t>BRD-05</t>
+        </is>
+      </c>
+      <c r="B74" s="12" t="inlineStr">
+        <is>
+          <t>FitGap</t>
+        </is>
+      </c>
+      <c r="C74" s="12" t="inlineStr">
+        <is>
+          <t>Accounting Disbursement ACSL BRD vs OOTB vs Best Practice</t>
+        </is>
+      </c>
+      <c r="D74" s="12" t="inlineStr">
+        <is>
+          <t>BIBS_FitGap_BRD-05_Accounting_Disbursement_ACSL_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+        </is>
+      </c>
+      <c r="E74" s="12" t="inlineStr">
+        <is>
+          <t>XLSX</t>
+        </is>
+      </c>
+      <c r="F74" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G74" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H74" s="12" t="inlineStr">
+        <is>
+          <t>BIBS Product Owner</t>
+        </is>
+      </c>
+      <c r="I74" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="J74" s="22" t="inlineStr">
+        <is>
+          <t>Issued for BDOI review</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="12" t="inlineStr">
+        <is>
+          <t>BRD-07</t>
+        </is>
+      </c>
+      <c r="B75" s="12" t="inlineStr">
+        <is>
+          <t>FitGap</t>
+        </is>
+      </c>
+      <c r="C75" s="12" t="inlineStr">
+        <is>
+          <t>Claims BRD vs OOTB vs Best Practice</t>
+        </is>
+      </c>
+      <c r="D75" s="12" t="inlineStr">
+        <is>
+          <t>BIBS_FitGap_BRD-07_Claims_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+        </is>
+      </c>
+      <c r="E75" s="12" t="inlineStr">
+        <is>
+          <t>XLSX</t>
+        </is>
+      </c>
+      <c r="F75" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G75" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H75" s="12" t="inlineStr">
+        <is>
+          <t>BIBS Product Owner</t>
+        </is>
+      </c>
+      <c r="I75" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="J75" s="22" t="inlineStr">
+        <is>
+          <t>Issued for BDOI review</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="12" t="inlineStr">
+        <is>
+          <t>BRD-08</t>
+        </is>
+      </c>
+      <c r="B76" s="12" t="inlineStr">
+        <is>
+          <t>FitGap</t>
+        </is>
+      </c>
+      <c r="C76" s="12" t="inlineStr">
+        <is>
+          <t>Employee Benefits BRD vs OOTB vs Best Practice</t>
+        </is>
+      </c>
+      <c r="D76" s="12" t="inlineStr">
+        <is>
+          <t>BIBS_FitGap_BRD-08_Employee_Benefits_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+        </is>
+      </c>
+      <c r="E76" s="12" t="inlineStr">
+        <is>
+          <t>XLSX</t>
+        </is>
+      </c>
+      <c r="F76" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G76" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H76" s="12" t="inlineStr">
+        <is>
+          <t>BIBS Product Owner</t>
+        </is>
+      </c>
+      <c r="I76" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="J76" s="22" t="inlineStr">
+        <is>
+          <t>Issued for BDOI review</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="12" t="inlineStr">
+        <is>
+          <t>BRD-09</t>
+        </is>
+      </c>
+      <c r="B77" s="12" t="inlineStr">
+        <is>
+          <t>FitGap</t>
+        </is>
+      </c>
+      <c r="C77" s="12" t="inlineStr">
+        <is>
+          <t>Customer Servicing Facility BRD vs OOTB vs Best Practice</t>
+        </is>
+      </c>
+      <c r="D77" s="12" t="inlineStr">
+        <is>
+          <t>BIBS_FitGap_BRD-09_Customer_Servicing_Facility_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+        </is>
+      </c>
+      <c r="E77" s="12" t="inlineStr">
+        <is>
+          <t>XLSX</t>
+        </is>
+      </c>
+      <c r="F77" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G77" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H77" s="12" t="inlineStr">
+        <is>
+          <t>BIBS Product Owner</t>
+        </is>
+      </c>
+      <c r="I77" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="J77" s="22" t="inlineStr">
+        <is>
+          <t>Issued for BDOI review</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="12" t="inlineStr">
+        <is>
+          <t>BRD-10</t>
+        </is>
+      </c>
+      <c r="B78" s="12" t="inlineStr">
+        <is>
+          <t>FitGap</t>
+        </is>
+      </c>
+      <c r="C78" s="12" t="inlineStr">
+        <is>
+          <t>Sanction Screening BRD vs OOTB vs Best Practice</t>
+        </is>
+      </c>
+      <c r="D78" s="12" t="inlineStr">
+        <is>
+          <t>BIBS_FitGap_BRD-10_Sanction_Screening_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+        </is>
+      </c>
+      <c r="E78" s="12" t="inlineStr">
+        <is>
+          <t>XLSX</t>
+        </is>
+      </c>
+      <c r="F78" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G78" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H78" s="12" t="inlineStr">
+        <is>
+          <t>BIBS Product Owner</t>
+        </is>
+      </c>
+      <c r="I78" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="J78" s="22" t="inlineStr">
+        <is>
+          <t>Issued for BDOI review</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="12" t="inlineStr">
+        <is>
+          <t>BRD-12</t>
+        </is>
+      </c>
+      <c r="B79" s="12" t="inlineStr">
+        <is>
+          <t>FitGap</t>
+        </is>
+      </c>
+      <c r="C79" s="12" t="inlineStr">
+        <is>
+          <t>Submitted Policies BRD vs OOTB vs Best Practice</t>
+        </is>
+      </c>
+      <c r="D79" s="12" t="inlineStr">
+        <is>
+          <t>BIBS_FitGap_BRD-12_Submitted_Policies_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+        </is>
+      </c>
+      <c r="E79" s="12" t="inlineStr">
+        <is>
+          <t>XLSX</t>
+        </is>
+      </c>
+      <c r="F79" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G79" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H79" s="12" t="inlineStr">
+        <is>
+          <t>BIBS Product Owner</t>
+        </is>
+      </c>
+      <c r="I79" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="J79" s="22" t="inlineStr">
+        <is>
+          <t>Issued for BDOI review</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="12" t="inlineStr">
+        <is>
+          <t>BRD-13</t>
+        </is>
+      </c>
+      <c r="B80" s="12" t="inlineStr">
+        <is>
+          <t>FitGap</t>
+        </is>
+      </c>
+      <c r="C80" s="12" t="inlineStr">
+        <is>
+          <t>Data Migration BRD vs OOTB vs Best Practice</t>
+        </is>
+      </c>
+      <c r="D80" s="12" t="inlineStr">
+        <is>
+          <t>BIBS_FitGap_BRD-13_Data_Migration_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+        </is>
+      </c>
+      <c r="E80" s="12" t="inlineStr">
+        <is>
+          <t>XLSX</t>
+        </is>
+      </c>
+      <c r="F80" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G80" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H80" s="12" t="inlineStr">
+        <is>
+          <t>BIBS Product Owner</t>
+        </is>
+      </c>
+      <c r="I80" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="J80" s="22" t="inlineStr">
+        <is>
+          <t>Issued for BDOI review</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J69"/>
+  <autoFilter ref="A4:J80"/>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:J569">
+  <conditionalFormatting sqref="A5:J580">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J5:J569" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
+    <dataValidation sqref="J5:J580" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
       <formula1>'Lists'!$A$2:$A$5</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Access matrix of every BRD pack from the permissions, group profiles, menus and server checks
New pack_access builder (document key ACX) wired into build_pack.py and the
Remittance and Claims pack builder: group profile x screen x action with the
permission each action asks for, the group profiles, the menu of each
persona and the service operations of the pack. Issued as
BIBS_Access_BRD-xx_..._Access_Matrix_v1.0.xlsx in the six packs and listed
in each How to Read note and in the Document Register. The Remittance and
Claims developer specifications now include the settings, claim handling
and checklist services.
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Common/BIBS_Register_BRD-00_Document_Register_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Common/BIBS_Register_BRD-00_Document_Register_v1.0.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'README'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Register'!$A$4:$J$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Register'!$A$4:$J$117</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Register'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Lists'!$1:$1</definedName>
   </definedNames>
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="D21" s="14" t="n">
-        <v>107</v>
+        <v>113</v>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
@@ -1053,7 +1053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J111"/>
+  <dimension ref="A1:J117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1154,27 +1154,27 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>BPS</t>
+          <t>Access</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>User Access Process and Storyboards</t>
+          <t>Access Matrix</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>BIBS_BPS-BDOI_BRD-11_User_Access_Process_and_Storyboards_v1.6</t>
+          <t>BIBS_Access_BRD-11_Access_Matrix_v1.0</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G5" s="12" t="inlineStr">
@@ -1206,27 +1206,27 @@
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>BPS</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>Change Request Register</t>
+          <t>User Access Process and Storyboards</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>BIBS_CR_BRD-11_Change_Request_Register_v1.3</t>
+          <t>BIBS_BPS-BDOI_BRD-11_User_Access_Process_and_Storyboards_v1.6</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="G6" s="12" t="inlineStr">
@@ -1263,12 +1263,12 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>Effort Estimate</t>
+          <t>Change Request Register</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>BIBS_CR_BRD-11_Effort_Estimate_v1.3</t>
+          <t>BIBS_CR_BRD-11_Change_Request_Register_v1.3</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -1310,17 +1310,17 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>DDI</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>User Access Data Dictionary</t>
+          <t>Effort Estimate</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>BIBS_DDI-BDOI_BRD-11_User_Access_Data_Dictionary_v1.0</t>
+          <t>BIBS_CR_BRD-11_Effort_Estimate_v1.3</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="G8" s="12" t="inlineStr">
@@ -1362,22 +1362,22 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>DDI</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>User Access Developer Specification</t>
+          <t>User Access Data Dictionary</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>BIBS_DSP-BDOI_BRD-11_User_Access_Developer_Specification_v1.0</t>
+          <t>BIBS_DDI-BDOI_BRD-11_User_Access_Data_Dictionary_v1.0</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
@@ -1414,17 +1414,17 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>FRS</t>
+          <t>DSP</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>User Access Maintenance</t>
+          <t>User Access Developer Specification</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FRS-BDOI_BRD-11_User_Access_Maintenance_v1.6</t>
+          <t>BIBS_DSP-BDOI_BRD-11_User_Access_Developer_Specification_v1.0</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
@@ -1434,7 +1434,7 @@
       </c>
       <c r="F10" s="12" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G10" s="12" t="inlineStr">
@@ -1466,27 +1466,27 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>FitGap</t>
+          <t>FRS</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>BRD vs OOTB vs Best Practice</t>
+          <t>User Access Maintenance</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FitGap_BRD-11_BRD_vs_OOTB_vs_Best_Practice_v1.3</t>
+          <t>BIBS_FRS-BDOI_BRD-11_User_Access_Maintenance_v1.6</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
@@ -1518,17 +1518,17 @@
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>ICD</t>
+          <t>FitGap</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>Interface Test Pack</t>
+          <t>BRD vs OOTB vs Best Practice</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>BIBS_ICD-BDOI_BRD-11_Interface_Test_Pack_v1.1</t>
+          <t>BIBS_FitGap_BRD-11_BRD_vs_OOTB_vs_Best_Practice_v1.3</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="G12" s="12" t="inlineStr">
@@ -1575,17 +1575,17 @@
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>SCIM OpenAPI</t>
+          <t>Interface Test Pack</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>BIBS_ICD-BDOI_BRD-11_SCIM_OpenAPI_v1.1</t>
+          <t>BIBS_ICD-BDOI_BRD-11_Interface_Test_Pack_v1.1</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>YAML</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
@@ -1627,17 +1627,17 @@
       </c>
       <c r="C14" s="12" t="inlineStr">
         <is>
-          <t>User Access Interface Specification</t>
+          <t>SCIM OpenAPI</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>BIBS_ICD-BDOI_BRD-11_User_Access_Interface_Specification_v1.1</t>
+          <t>BIBS_ICD-BDOI_BRD-11_SCIM_OpenAPI_v1.1</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>YAML</t>
         </is>
       </c>
       <c r="F14" s="12" t="inlineStr">
@@ -1674,27 +1674,27 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Inputs</t>
+          <t>ICD</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>Business Unit Requirements Collection</t>
+          <t>User Access Interface Specification</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>BIBS_Inputs_BRD-11_Business_Unit_Requirements_Collection_v1.3</t>
+          <t>BIBS_ICD-BDOI_BRD-11_User_Access_Interface_Specification_v1.1</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G15" s="12" t="inlineStr">
@@ -1726,27 +1726,27 @@
       </c>
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t>README</t>
+          <t>Inputs</t>
         </is>
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>How to Read this Pack</t>
+          <t>Business Unit Requirements Collection</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>BIBS_Inputs_BRD-11_How_to_Read_this_Pack_v1.0</t>
+          <t>BIBS_Inputs_BRD-11_Business_Unit_Requirements_Collection_v1.3</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F16" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="G16" s="12" t="inlineStr">
@@ -1778,17 +1778,17 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>RNO</t>
+          <t>README</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>User Access Reports Notifications Outputs</t>
+          <t>How to Read this Pack</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>BIBS_RNO-BDOI_BRD-11_User_Access_Reports_Notifications_Outputs_v1.6</t>
+          <t>BIBS_Inputs_BRD-11_How_to_Read_this_Pack_v1.0</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G17" s="12" t="inlineStr">
@@ -1830,27 +1830,27 @@
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>RTM</t>
+          <t>RNO</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>Test Cases and Traceability</t>
+          <t>User Access Reports Notifications Outputs</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>BIBS_RTM_BRD-11_Test_Cases_and_Traceability_v1.3</t>
+          <t>BIBS_RNO-BDOI_BRD-11_User_Access_Reports_Notifications_Outputs_v1.6</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="G18" s="12" t="inlineStr">
@@ -1882,17 +1882,17 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>RTM</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>Business Unit Walkthrough Users</t>
+          <t>Test Cases and Traceability</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>BIBS_UAT_BRD-11_Business_Unit_Walkthrough_Users_v1.3</t>
+          <t>BIBS_RTM_BRD-11_Test_Cases_and_Traceability_v1.3</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
@@ -1934,17 +1934,17 @@
       </c>
       <c r="B20" s="12" t="inlineStr">
         <is>
-          <t>USR</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>User Access User Stories</t>
+          <t>Business Unit Walkthrough Users</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>BIBS_USR-BDOI_BRD-11_User_Access_User_Stories_v1.0</t>
+          <t>BIBS_UAT_BRD-11_Business_Unit_Walkthrough_Users_v1.3</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="F20" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="G20" s="12" t="inlineStr">
@@ -1986,27 +1986,27 @@
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>UXD</t>
+          <t>USR</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>User Access UX Design</t>
+          <t>User Access User Stories</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>BIBS_UXD-BDOI_BRD-11_User_Access_UX_Design_v1.6</t>
+          <t>BIBS_USR-BDOI_BRD-11_User_Access_User_Stories_v1.0</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G21" s="12" t="inlineStr">
@@ -2033,22 +2033,22 @@
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>BRD-03</t>
+          <t>BRD-11</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>BPS</t>
+          <t>UXD</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>Product Maintenance Process and Storyboards</t>
+          <t>User Access UX Design</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>BIBS_BPS-BDOI_BRD-03_Product_Maintenance_Process_and_Storyboards_v1.7</t>
+          <t>BIBS_UXD-BDOI_BRD-11_User_Access_UX_Design_v1.6</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -2058,17 +2058,17 @@
       </c>
       <c r="F22" s="12" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="G22" s="12" t="inlineStr">
         <is>
-          <t>17 Oct 2026</t>
+          <t>16 Oct 2026</t>
         </is>
       </c>
       <c r="H22" s="12" t="inlineStr">
         <is>
-          <t>BDOI Product Owner, Product Maintenance</t>
+          <t>BDOI Product Owner, User Access</t>
         </is>
       </c>
       <c r="I22" s="12" t="inlineStr">
@@ -2090,17 +2090,17 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>Access</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>Change Request Register</t>
+          <t>Access Matrix</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>BIBS_CR_BRD-03_Change_Request_Register_v1.4</t>
+          <t>BIBS_Access_BRD-03_Access_Matrix_v1.0</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
@@ -2110,12 +2110,12 @@
       </c>
       <c r="F23" s="12" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G23" s="12" t="inlineStr">
         <is>
-          <t>16 Oct 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="H23" s="12" t="inlineStr">
@@ -2142,32 +2142,32 @@
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>BPS</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
-          <t>Effort Estimate</t>
+          <t>Product Maintenance Process and Storyboards</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>BIBS_CR_BRD-03_Effort_Estimate_v1.4</t>
+          <t>BIBS_BPS-BDOI_BRD-03_Product_Maintenance_Process_and_Storyboards_v1.7</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F24" s="12" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="G24" s="12" t="inlineStr">
         <is>
-          <t>16 Oct 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="H24" s="12" t="inlineStr">
@@ -2194,17 +2194,17 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>DDI</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>Product Maintenance Data Dictionary</t>
+          <t>Change Request Register</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>BIBS_DDI-BDOI_BRD-03_Product_Maintenance_Data_Dictionary_v1.2</t>
+          <t>BIBS_CR_BRD-03_Change_Request_Register_v1.4</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
@@ -2214,12 +2214,12 @@
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="G25" s="12" t="inlineStr">
         <is>
-          <t>17 Oct 2026</t>
+          <t>16 Oct 2026</t>
         </is>
       </c>
       <c r="H25" s="12" t="inlineStr">
@@ -2246,22 +2246,22 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>Product Maintenance Developer Specification</t>
+          <t>Effort Estimate</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>BIBS_DSP-BDOI_BRD-03_Product_Maintenance_Developer_Specification_v1.4</t>
+          <t>BIBS_CR_BRD-03_Effort_Estimate_v1.4</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="G26" s="12" t="inlineStr">
         <is>
-          <t>17 Oct 2026</t>
+          <t>16 Oct 2026</t>
         </is>
       </c>
       <c r="H26" s="12" t="inlineStr">
@@ -2298,27 +2298,27 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>FRS</t>
+          <t>DDI</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>Product Maintenance</t>
+          <t>Product Maintenance Data Dictionary</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FRS-BDOI_BRD-03_Product_Maintenance_v1.7</t>
+          <t>BIBS_DDI-BDOI_BRD-03_Product_Maintenance_Data_Dictionary_v1.2</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F27" s="12" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="G27" s="12" t="inlineStr">
@@ -2350,22 +2350,22 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>FitGap</t>
+          <t>DSP</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>BRD vs OOTB vs Best Practice</t>
+          <t>Product Maintenance Developer Specification</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FitGap_BRD-03_BRD_vs_OOTB_vs_Best_Practice_v1.4</t>
+          <t>BIBS_DSP-BDOI_BRD-03_Product_Maintenance_Developer_Specification_v1.4</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G28" s="12" t="inlineStr">
         <is>
-          <t>16 Oct 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="H28" s="12" t="inlineStr">
@@ -2402,17 +2402,17 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>ICD</t>
+          <t>FRS</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>Product Maintenance Interface Specification</t>
+          <t>Product Maintenance</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>BIBS_ICD-BDOI_BRD-03_Product_Maintenance_Interface_Specification_v1.0</t>
+          <t>BIBS_FRS-BDOI_BRD-03_Product_Maintenance_v1.7</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
@@ -2422,12 +2422,12 @@
       </c>
       <c r="F29" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="G29" s="12" t="inlineStr">
         <is>
-          <t>16 Oct 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="H29" s="12" t="inlineStr">
@@ -2454,17 +2454,17 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>Inputs</t>
+          <t>FitGap</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>Business Unit Requirements Collection</t>
+          <t>BRD vs OOTB vs Best Practice</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>BIBS_Inputs_BRD-03_Business_Unit_Requirements_Collection_v1.4</t>
+          <t>BIBS_FitGap_BRD-03_BRD_vs_OOTB_vs_Best_Practice_v1.4</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2506,17 +2506,17 @@
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>README</t>
+          <t>ICD</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>How to Read this Pack</t>
+          <t>Product Maintenance Interface Specification</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>BIBS_Inputs_BRD-03_How_to_Read_this_Pack_v1.0</t>
+          <t>BIBS_ICD-BDOI_BRD-03_Product_Maintenance_Interface_Specification_v1.0</t>
         </is>
       </c>
       <c r="E31" s="12" t="inlineStr">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="G31" s="12" t="inlineStr">
         <is>
-          <t>17 Oct 2026</t>
+          <t>16 Oct 2026</t>
         </is>
       </c>
       <c r="H31" s="12" t="inlineStr">
@@ -2558,32 +2558,32 @@
       </c>
       <c r="B32" s="12" t="inlineStr">
         <is>
-          <t>RNO</t>
+          <t>Inputs</t>
         </is>
       </c>
       <c r="C32" s="12" t="inlineStr">
         <is>
-          <t>Product Maintenance Reports Notifications Outputs</t>
+          <t>Business Unit Requirements Collection</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>BIBS_RNO-BDOI_BRD-03_Product_Maintenance_Reports_Notifications_Outputs_v1.7</t>
+          <t>BIBS_Inputs_BRD-03_Business_Unit_Requirements_Collection_v1.4</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F32" s="12" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="G32" s="12" t="inlineStr">
         <is>
-          <t>17 Oct 2026</t>
+          <t>16 Oct 2026</t>
         </is>
       </c>
       <c r="H32" s="12" t="inlineStr">
@@ -2610,32 +2610,32 @@
       </c>
       <c r="B33" s="12" t="inlineStr">
         <is>
-          <t>RTM</t>
+          <t>README</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
-          <t>Test Cases and Traceability</t>
+          <t>How to Read this Pack</t>
         </is>
       </c>
       <c r="D33" s="12" t="inlineStr">
         <is>
-          <t>BIBS_RTM_BRD-03_Test_Cases_and_Traceability_v1.4</t>
+          <t>BIBS_Inputs_BRD-03_How_to_Read_this_Pack_v1.0</t>
         </is>
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F33" s="12" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G33" s="12" t="inlineStr">
         <is>
-          <t>16 Oct 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="H33" s="12" t="inlineStr">
@@ -2662,32 +2662,32 @@
       </c>
       <c r="B34" s="12" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>RNO</t>
         </is>
       </c>
       <c r="C34" s="12" t="inlineStr">
         <is>
-          <t>Business Unit Walkthrough Users</t>
+          <t>Product Maintenance Reports Notifications Outputs</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
         <is>
-          <t>BIBS_UAT_BRD-03_Business_Unit_Walkthrough_Users_v1.4</t>
+          <t>BIBS_RNO-BDOI_BRD-03_Product_Maintenance_Reports_Notifications_Outputs_v1.7</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F34" s="12" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="G34" s="12" t="inlineStr">
         <is>
-          <t>16 Oct 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="H34" s="12" t="inlineStr">
@@ -2714,17 +2714,17 @@
       </c>
       <c r="B35" s="12" t="inlineStr">
         <is>
-          <t>USR</t>
+          <t>RTM</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
-          <t>Product Maintenance User Stories</t>
+          <t>Test Cases and Traceability</t>
         </is>
       </c>
       <c r="D35" s="12" t="inlineStr">
         <is>
-          <t>BIBS_USR-BDOI_BRD-03_Product_Maintenance_User_Stories_v1.3</t>
+          <t>BIBS_RTM_BRD-03_Test_Cases_and_Traceability_v1.4</t>
         </is>
       </c>
       <c r="E35" s="12" t="inlineStr">
@@ -2734,12 +2734,12 @@
       </c>
       <c r="F35" s="12" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="G35" s="12" t="inlineStr">
         <is>
-          <t>17 Oct 2026</t>
+          <t>16 Oct 2026</t>
         </is>
       </c>
       <c r="H35" s="12" t="inlineStr">
@@ -2766,32 +2766,32 @@
       </c>
       <c r="B36" s="12" t="inlineStr">
         <is>
-          <t>UXD</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="C36" s="12" t="inlineStr">
         <is>
-          <t>Product Maintenance UX Design</t>
+          <t>Business Unit Walkthrough Users</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
         <is>
-          <t>BIBS_UXD-BDOI_BRD-03_Product_Maintenance_UX_Design_v1.8</t>
+          <t>BIBS_UAT_BRD-03_Business_Unit_Walkthrough_Users_v1.4</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F36" s="12" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="G36" s="12" t="inlineStr">
         <is>
-          <t>17 Oct 2026</t>
+          <t>16 Oct 2026</t>
         </is>
       </c>
       <c r="H36" s="12" t="inlineStr">
@@ -2813,27 +2813,27 @@
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
         <is>
-          <t>BRD-06</t>
+          <t>BRD-03</t>
         </is>
       </c>
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>BPS</t>
+          <t>USR</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>Renewal Process and Storyboards</t>
+          <t>Product Maintenance User Stories</t>
         </is>
       </c>
       <c r="D37" s="12" t="inlineStr">
         <is>
-          <t>BIBS_BPS-BDOI_BRD-06_Renewal_Process_and_Storyboards_v1.3</t>
+          <t>BIBS_USR-BDOI_BRD-03_Product_Maintenance_User_Stories_v1.3</t>
         </is>
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F37" s="12" t="inlineStr">
@@ -2843,12 +2843,12 @@
       </c>
       <c r="G37" s="12" t="inlineStr">
         <is>
-          <t>16 Oct 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="H37" s="12" t="inlineStr">
         <is>
-          <t>BDOI Product Owner, Renewal</t>
+          <t>BDOI Product Owner, Product Maintenance</t>
         </is>
       </c>
       <c r="I37" s="12" t="inlineStr">
@@ -2865,42 +2865,42 @@
     <row r="38">
       <c r="A38" s="12" t="inlineStr">
         <is>
-          <t>BRD-06</t>
+          <t>BRD-03</t>
         </is>
       </c>
       <c r="B38" s="12" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>UXD</t>
         </is>
       </c>
       <c r="C38" s="12" t="inlineStr">
         <is>
-          <t>Change Request Register</t>
+          <t>Product Maintenance UX Design</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
         <is>
-          <t>BIBS_CR_BRD-06_Change_Request_Register_v1.1</t>
+          <t>BIBS_UXD-BDOI_BRD-03_Product_Maintenance_UX_Design_v1.8</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F38" s="12" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="G38" s="12" t="inlineStr">
         <is>
-          <t>16 Oct 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="H38" s="12" t="inlineStr">
         <is>
-          <t>BDOI Product Owner, Renewal</t>
+          <t>BDOI Product Owner, Product Maintenance</t>
         </is>
       </c>
       <c r="I38" s="12" t="inlineStr">
@@ -2922,17 +2922,17 @@
       </c>
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>Access</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr">
         <is>
-          <t>Effort Estimate</t>
+          <t>Access Matrix</t>
         </is>
       </c>
       <c r="D39" s="12" t="inlineStr">
         <is>
-          <t>BIBS_CR_BRD-06_Effort_Estimate_v1.1</t>
+          <t>BIBS_Access_BRD-06_Access_Matrix_v1.0</t>
         </is>
       </c>
       <c r="E39" s="12" t="inlineStr">
@@ -2942,7 +2942,7 @@
       </c>
       <c r="F39" s="12" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G39" s="12" t="inlineStr">
@@ -2974,27 +2974,27 @@
       </c>
       <c r="B40" s="12" t="inlineStr">
         <is>
-          <t>DDI</t>
+          <t>BPS</t>
         </is>
       </c>
       <c r="C40" s="12" t="inlineStr">
         <is>
-          <t>Renewal Data Dictionary</t>
+          <t>Renewal Process and Storyboards</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
         <is>
-          <t>BIBS_DDI-BDOI_BRD-06_Renewal_Data_Dictionary_v1.0</t>
+          <t>BIBS_BPS-BDOI_BRD-06_Renewal_Process_and_Storyboards_v1.3</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F40" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="G40" s="12" t="inlineStr">
@@ -3026,27 +3026,27 @@
       </c>
       <c r="B41" s="12" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr">
         <is>
-          <t>Renewal Developer Specification</t>
+          <t>Change Request Register</t>
         </is>
       </c>
       <c r="D41" s="12" t="inlineStr">
         <is>
-          <t>BIBS_DSP-BDOI_BRD-06_Renewal_Developer_Specification_v1.0</t>
+          <t>BIBS_CR_BRD-06_Change_Request_Register_v1.1</t>
         </is>
       </c>
       <c r="E41" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F41" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G41" s="12" t="inlineStr">
@@ -3078,27 +3078,27 @@
       </c>
       <c r="B42" s="12" t="inlineStr">
         <is>
-          <t>FRS</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C42" s="12" t="inlineStr">
         <is>
-          <t>Renewal</t>
+          <t>Effort Estimate</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FRS-BDOI_BRD-06_Renewal_v1.3</t>
+          <t>BIBS_CR_BRD-06_Effort_Estimate_v1.1</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F42" s="12" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G42" s="12" t="inlineStr">
@@ -3130,17 +3130,17 @@
       </c>
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t>FitGap</t>
+          <t>DDI</t>
         </is>
       </c>
       <c r="C43" s="12" t="inlineStr">
         <is>
-          <t>BRD vs OOTB vs Best Practice</t>
+          <t>Renewal Data Dictionary</t>
         </is>
       </c>
       <c r="D43" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FitGap_BRD-06_BRD_vs_OOTB_vs_Best_Practice_v1.1</t>
+          <t>BIBS_DDI-BDOI_BRD-06_Renewal_Data_Dictionary_v1.0</t>
         </is>
       </c>
       <c r="E43" s="12" t="inlineStr">
@@ -3150,7 +3150,7 @@
       </c>
       <c r="F43" s="12" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G43" s="12" t="inlineStr">
@@ -3182,17 +3182,17 @@
       </c>
       <c r="B44" s="12" t="inlineStr">
         <is>
-          <t>ICD</t>
+          <t>DSP</t>
         </is>
       </c>
       <c r="C44" s="12" t="inlineStr">
         <is>
-          <t>Renewal Interface Specification</t>
+          <t>Renewal Developer Specification</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
-          <t>BIBS_ICD-BDOI_BRD-06_Renewal_Interface_Specification_v1.0</t>
+          <t>BIBS_DSP-BDOI_BRD-06_Renewal_Developer_Specification_v1.0</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -3234,27 +3234,27 @@
       </c>
       <c r="B45" s="12" t="inlineStr">
         <is>
-          <t>Inputs</t>
+          <t>FRS</t>
         </is>
       </c>
       <c r="C45" s="12" t="inlineStr">
         <is>
-          <t>Business Unit Requirements Collection</t>
+          <t>Renewal</t>
         </is>
       </c>
       <c r="D45" s="12" t="inlineStr">
         <is>
-          <t>BIBS_Inputs_BRD-06_Business_Unit_Requirements_Collection_v1.1</t>
+          <t>BIBS_FRS-BDOI_BRD-06_Renewal_v1.3</t>
         </is>
       </c>
       <c r="E45" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F45" s="12" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="G45" s="12" t="inlineStr">
@@ -3286,27 +3286,27 @@
       </c>
       <c r="B46" s="12" t="inlineStr">
         <is>
-          <t>README</t>
+          <t>FitGap</t>
         </is>
       </c>
       <c r="C46" s="12" t="inlineStr">
         <is>
-          <t>How to Read this Pack</t>
+          <t>BRD vs OOTB vs Best Practice</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
         <is>
-          <t>BIBS_Inputs_BRD-06_How_to_Read_this_Pack_v1.0</t>
+          <t>BIBS_FitGap_BRD-06_BRD_vs_OOTB_vs_Best_Practice_v1.1</t>
         </is>
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F46" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G46" s="12" t="inlineStr">
@@ -3338,17 +3338,17 @@
       </c>
       <c r="B47" s="12" t="inlineStr">
         <is>
-          <t>RNO</t>
+          <t>ICD</t>
         </is>
       </c>
       <c r="C47" s="12" t="inlineStr">
         <is>
-          <t>Renewal Reports Notifications Outputs</t>
+          <t>Renewal Interface Specification</t>
         </is>
       </c>
       <c r="D47" s="12" t="inlineStr">
         <is>
-          <t>BIBS_RNO-BDOI_BRD-06_Renewal_Reports_Notifications_Outputs_v1.3</t>
+          <t>BIBS_ICD-BDOI_BRD-06_Renewal_Interface_Specification_v1.0</t>
         </is>
       </c>
       <c r="E47" s="12" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="F47" s="12" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G47" s="12" t="inlineStr">
@@ -3390,17 +3390,17 @@
       </c>
       <c r="B48" s="12" t="inlineStr">
         <is>
-          <t>RTM</t>
+          <t>Inputs</t>
         </is>
       </c>
       <c r="C48" s="12" t="inlineStr">
         <is>
-          <t>Test Cases and Traceability</t>
+          <t>Business Unit Requirements Collection</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
         <is>
-          <t>BIBS_RTM_BRD-06_Test_Cases_and_Traceability_v1.1</t>
+          <t>BIBS_Inputs_BRD-06_Business_Unit_Requirements_Collection_v1.1</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
@@ -3442,27 +3442,27 @@
       </c>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>README</t>
         </is>
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>Business Unit Walkthrough Users</t>
+          <t>How to Read this Pack</t>
         </is>
       </c>
       <c r="D49" s="12" t="inlineStr">
         <is>
-          <t>BIBS_UAT_BRD-06_Business_Unit_Walkthrough_Users_v1.1</t>
+          <t>BIBS_Inputs_BRD-06_How_to_Read_this_Pack_v1.0</t>
         </is>
       </c>
       <c r="E49" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F49" s="12" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G49" s="12" t="inlineStr">
@@ -3494,27 +3494,27 @@
       </c>
       <c r="B50" s="12" t="inlineStr">
         <is>
-          <t>USR</t>
+          <t>RNO</t>
         </is>
       </c>
       <c r="C50" s="12" t="inlineStr">
         <is>
-          <t>Renewal User Stories</t>
+          <t>Renewal Reports Notifications Outputs</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
         <is>
-          <t>BIBS_USR-BDOI_BRD-06_Renewal_User_Stories_v1.0</t>
+          <t>BIBS_RNO-BDOI_BRD-06_Renewal_Reports_Notifications_Outputs_v1.3</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F50" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="G50" s="12" t="inlineStr">
@@ -3546,27 +3546,27 @@
       </c>
       <c r="B51" s="12" t="inlineStr">
         <is>
-          <t>UXD</t>
+          <t>RTM</t>
         </is>
       </c>
       <c r="C51" s="12" t="inlineStr">
         <is>
-          <t>Renewal UX Design</t>
+          <t>Test Cases and Traceability</t>
         </is>
       </c>
       <c r="D51" s="12" t="inlineStr">
         <is>
-          <t>BIBS_UXD-BDOI_BRD-06_Renewal_UX_Design_v1.3</t>
+          <t>BIBS_RTM_BRD-06_Test_Cases_and_Traceability_v1.1</t>
         </is>
       </c>
       <c r="E51" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F51" s="12" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G51" s="12" t="inlineStr">
@@ -3593,32 +3593,32 @@
     <row r="52">
       <c r="A52" s="12" t="inlineStr">
         <is>
-          <t>BRD-02</t>
+          <t>BRD-06</t>
         </is>
       </c>
       <c r="B52" s="12" t="inlineStr">
         <is>
-          <t>BPS</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="C52" s="12" t="inlineStr">
         <is>
-          <t>Operations Cashiering Process and Storyboards</t>
+          <t>Business Unit Walkthrough Users</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
         <is>
-          <t>BIBS_BPS-BDOI_BRD-02_Operations_Cashiering_Process_and_Storyboards_v3.4</t>
+          <t>BIBS_UAT_BRD-06_Business_Unit_Walkthrough_Users_v1.1</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F52" s="12" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G52" s="12" t="inlineStr">
@@ -3628,7 +3628,7 @@
       </c>
       <c r="H52" s="12" t="inlineStr">
         <is>
-          <t>BDOI Product Owner, Operations</t>
+          <t>BDOI Product Owner, Renewal</t>
         </is>
       </c>
       <c r="I52" s="12" t="inlineStr">
@@ -3645,22 +3645,22 @@
     <row r="53">
       <c r="A53" s="12" t="inlineStr">
         <is>
-          <t>BRD-02</t>
+          <t>BRD-06</t>
         </is>
       </c>
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>USR</t>
         </is>
       </c>
       <c r="C53" s="12" t="inlineStr">
         <is>
-          <t>Change Request Register</t>
+          <t>Renewal User Stories</t>
         </is>
       </c>
       <c r="D53" s="12" t="inlineStr">
         <is>
-          <t>BIBS_CR_BRD-02_Change_Request_Register_v1.1</t>
+          <t>BIBS_USR-BDOI_BRD-06_Renewal_User_Stories_v1.0</t>
         </is>
       </c>
       <c r="E53" s="12" t="inlineStr">
@@ -3670,7 +3670,7 @@
       </c>
       <c r="F53" s="12" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G53" s="12" t="inlineStr">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="H53" s="12" t="inlineStr">
         <is>
-          <t>BDOI Product Owner, Operations</t>
+          <t>BDOI Product Owner, Renewal</t>
         </is>
       </c>
       <c r="I53" s="12" t="inlineStr">
@@ -3697,32 +3697,32 @@
     <row r="54">
       <c r="A54" s="12" t="inlineStr">
         <is>
-          <t>BRD-02</t>
+          <t>BRD-06</t>
         </is>
       </c>
       <c r="B54" s="12" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>UXD</t>
         </is>
       </c>
       <c r="C54" s="12" t="inlineStr">
         <is>
-          <t>Effort Estimate</t>
+          <t>Renewal UX Design</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
         <is>
-          <t>BIBS_CR_BRD-02_Effort_Estimate_v1.1</t>
+          <t>BIBS_UXD-BDOI_BRD-06_Renewal_UX_Design_v1.3</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F54" s="12" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="G54" s="12" t="inlineStr">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="H54" s="12" t="inlineStr">
         <is>
-          <t>BDOI Product Owner, Operations</t>
+          <t>BDOI Product Owner, Renewal</t>
         </is>
       </c>
       <c r="I54" s="12" t="inlineStr">
@@ -3754,17 +3754,17 @@
       </c>
       <c r="B55" s="12" t="inlineStr">
         <is>
-          <t>DDI</t>
+          <t>Access</t>
         </is>
       </c>
       <c r="C55" s="12" t="inlineStr">
         <is>
-          <t>Operations Cashiering Data Dictionary</t>
+          <t>Cashiering Access Matrix</t>
         </is>
       </c>
       <c r="D55" s="12" t="inlineStr">
         <is>
-          <t>BIBS_DDI-BDOI_BRD-02_Operations_Cashiering_Data_Dictionary_v1.0</t>
+          <t>BIBS_Access_BRD-02_Cashiering_Access_Matrix_v1.0</t>
         </is>
       </c>
       <c r="E55" s="12" t="inlineStr">
@@ -3806,17 +3806,17 @@
       </c>
       <c r="B56" s="12" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>BPS</t>
         </is>
       </c>
       <c r="C56" s="12" t="inlineStr">
         <is>
-          <t>Operations Cashiering Developer Specification</t>
+          <t>Operations Cashiering Process and Storyboards</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
         <is>
-          <t>BIBS_DSP-BDOI_BRD-02_Operations_Cashiering_Developer_Specification_v1.0</t>
+          <t>BIBS_BPS-BDOI_BRD-02_Operations_Cashiering_Process_and_Storyboards_v3.4</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
@@ -3826,7 +3826,7 @@
       </c>
       <c r="F56" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="G56" s="12" t="inlineStr">
@@ -3858,27 +3858,27 @@
       </c>
       <c r="B57" s="12" t="inlineStr">
         <is>
-          <t>FRS</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C57" s="12" t="inlineStr">
         <is>
-          <t>Operations Cashiering</t>
+          <t>Change Request Register</t>
         </is>
       </c>
       <c r="D57" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FRS-BDOI_BRD-02_Operations_Cashiering_v3.4</t>
+          <t>BIBS_CR_BRD-02_Change_Request_Register_v1.1</t>
         </is>
       </c>
       <c r="E57" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F57" s="12" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G57" s="12" t="inlineStr">
@@ -3910,17 +3910,17 @@
       </c>
       <c r="B58" s="12" t="inlineStr">
         <is>
-          <t>FitGap</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C58" s="12" t="inlineStr">
         <is>
-          <t>BRD vs OOTB vs Best Practice</t>
+          <t>Effort Estimate</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FitGap_BRD-02_BRD_vs_OOTB_vs_Best_Practice_v1.1</t>
+          <t>BIBS_CR_BRD-02_Effort_Estimate_v1.1</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
@@ -3962,22 +3962,22 @@
       </c>
       <c r="B59" s="12" t="inlineStr">
         <is>
-          <t>ICD</t>
+          <t>DDI</t>
         </is>
       </c>
       <c r="C59" s="12" t="inlineStr">
         <is>
-          <t>Operations Cashiering Interface Specification</t>
+          <t>Operations Cashiering Data Dictionary</t>
         </is>
       </c>
       <c r="D59" s="12" t="inlineStr">
         <is>
-          <t>BIBS_ICD-BDOI_BRD-02_Operations_Cashiering_Interface_Specification_v1.0</t>
+          <t>BIBS_DDI-BDOI_BRD-02_Operations_Cashiering_Data_Dictionary_v1.0</t>
         </is>
       </c>
       <c r="E59" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F59" s="12" t="inlineStr">
@@ -4014,27 +4014,27 @@
       </c>
       <c r="B60" s="12" t="inlineStr">
         <is>
-          <t>Inputs</t>
+          <t>DSP</t>
         </is>
       </c>
       <c r="C60" s="12" t="inlineStr">
         <is>
-          <t>Business Unit Requirements Collection</t>
+          <t>Operations Cashiering Developer Specification</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
         <is>
-          <t>BIBS_Inputs_BRD-02_Business_Unit_Requirements_Collection_v1.1</t>
+          <t>BIBS_DSP-BDOI_BRD-02_Operations_Cashiering_Developer_Specification_v1.0</t>
         </is>
       </c>
       <c r="E60" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F60" s="12" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G60" s="12" t="inlineStr">
@@ -4066,17 +4066,17 @@
       </c>
       <c r="B61" s="12" t="inlineStr">
         <is>
-          <t>README</t>
+          <t>FRS</t>
         </is>
       </c>
       <c r="C61" s="12" t="inlineStr">
         <is>
-          <t>How to Read this Pack</t>
+          <t>Operations Cashiering</t>
         </is>
       </c>
       <c r="D61" s="12" t="inlineStr">
         <is>
-          <t>BIBS_Inputs_BRD-02_How_to_Read_this_Pack_v1.0</t>
+          <t>BIBS_FRS-BDOI_BRD-02_Operations_Cashiering_v3.4</t>
         </is>
       </c>
       <c r="E61" s="12" t="inlineStr">
@@ -4086,7 +4086,7 @@
       </c>
       <c r="F61" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="G61" s="12" t="inlineStr">
@@ -4118,27 +4118,27 @@
       </c>
       <c r="B62" s="12" t="inlineStr">
         <is>
-          <t>RNO</t>
+          <t>FitGap</t>
         </is>
       </c>
       <c r="C62" s="12" t="inlineStr">
         <is>
-          <t>Operations Cashiering Reports Notifications Outputs</t>
+          <t>BRD vs OOTB vs Best Practice</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
         <is>
-          <t>BIBS_RNO-BDOI_BRD-02_Operations_Cashiering_Reports_Notifications_Outputs_v3.4</t>
+          <t>BIBS_FitGap_BRD-02_BRD_vs_OOTB_vs_Best_Practice_v1.1</t>
         </is>
       </c>
       <c r="E62" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F62" s="12" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G62" s="12" t="inlineStr">
@@ -4170,27 +4170,27 @@
       </c>
       <c r="B63" s="12" t="inlineStr">
         <is>
-          <t>RTM</t>
+          <t>ICD</t>
         </is>
       </c>
       <c r="C63" s="12" t="inlineStr">
         <is>
-          <t>Test Cases and Traceability</t>
+          <t>Operations Cashiering Interface Specification</t>
         </is>
       </c>
       <c r="D63" s="12" t="inlineStr">
         <is>
-          <t>BIBS_RTM_BRD-02_Test_Cases_and_Traceability_v1.1</t>
+          <t>BIBS_ICD-BDOI_BRD-02_Operations_Cashiering_Interface_Specification_v1.0</t>
         </is>
       </c>
       <c r="E63" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F63" s="12" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G63" s="12" t="inlineStr">
@@ -4222,17 +4222,17 @@
       </c>
       <c r="B64" s="12" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>Inputs</t>
         </is>
       </c>
       <c r="C64" s="12" t="inlineStr">
         <is>
-          <t>Business Unit Walkthrough Users</t>
+          <t>Business Unit Requirements Collection</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
         <is>
-          <t>BIBS_UAT_BRD-02_Business_Unit_Walkthrough_Users_v1.1</t>
+          <t>BIBS_Inputs_BRD-02_Business_Unit_Requirements_Collection_v1.1</t>
         </is>
       </c>
       <c r="E64" s="12" t="inlineStr">
@@ -4274,22 +4274,22 @@
       </c>
       <c r="B65" s="12" t="inlineStr">
         <is>
-          <t>USR</t>
+          <t>README</t>
         </is>
       </c>
       <c r="C65" s="12" t="inlineStr">
         <is>
-          <t>Operations Cashiering User Stories</t>
+          <t>How to Read this Pack</t>
         </is>
       </c>
       <c r="D65" s="12" t="inlineStr">
         <is>
-          <t>BIBS_USR-BDOI_BRD-02_Operations_Cashiering_User_Stories_v1.0</t>
+          <t>BIBS_Inputs_BRD-02_How_to_Read_this_Pack_v1.0</t>
         </is>
       </c>
       <c r="E65" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F65" s="12" t="inlineStr">
@@ -4326,17 +4326,17 @@
       </c>
       <c r="B66" s="12" t="inlineStr">
         <is>
-          <t>UXD</t>
+          <t>RNO</t>
         </is>
       </c>
       <c r="C66" s="12" t="inlineStr">
         <is>
-          <t>Operations Cashiering UX Design</t>
+          <t>Operations Cashiering Reports Notifications Outputs</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
         <is>
-          <t>BIBS_UXD-BDOI_BRD-02_Operations_Cashiering_UX_Design_v3.4</t>
+          <t>BIBS_RNO-BDOI_BRD-02_Operations_Cashiering_Reports_Notifications_Outputs_v3.4</t>
         </is>
       </c>
       <c r="E66" s="12" t="inlineStr">
@@ -4378,32 +4378,32 @@
       </c>
       <c r="B67" s="12" t="inlineStr">
         <is>
-          <t>BPS</t>
+          <t>RTM</t>
         </is>
       </c>
       <c r="C67" s="12" t="inlineStr">
         <is>
-          <t>Operations Remittance Process and Storyboards</t>
+          <t>Test Cases and Traceability</t>
         </is>
       </c>
       <c r="D67" s="12" t="inlineStr">
         <is>
-          <t>BIBS_BPS-BDOI_BRD-02_Operations_Remittance_Process_and_Storyboards_v1.0</t>
+          <t>BIBS_RTM_BRD-02_Test_Cases_and_Traceability_v1.1</t>
         </is>
       </c>
       <c r="E67" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F67" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G67" s="12" t="inlineStr">
         <is>
-          <t>17 Oct 2026</t>
+          <t>16 Oct 2026</t>
         </is>
       </c>
       <c r="H67" s="12" t="inlineStr">
@@ -4430,17 +4430,17 @@
       </c>
       <c r="B68" s="12" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="C68" s="12" t="inlineStr">
         <is>
-          <t>Remittance Change Request Register</t>
+          <t>Business Unit Walkthrough Users</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
         <is>
-          <t>BIBS_CR_BRD-02_Remittance_Change_Request_Register_v1.0</t>
+          <t>BIBS_UAT_BRD-02_Business_Unit_Walkthrough_Users_v1.1</t>
         </is>
       </c>
       <c r="E68" s="12" t="inlineStr">
@@ -4450,12 +4450,12 @@
       </c>
       <c r="F68" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G68" s="12" t="inlineStr">
         <is>
-          <t>17 Oct 2026</t>
+          <t>16 Oct 2026</t>
         </is>
       </c>
       <c r="H68" s="12" t="inlineStr">
@@ -4482,17 +4482,17 @@
       </c>
       <c r="B69" s="12" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>USR</t>
         </is>
       </c>
       <c r="C69" s="12" t="inlineStr">
         <is>
-          <t>Remittance Effort Estimate</t>
+          <t>Operations Cashiering User Stories</t>
         </is>
       </c>
       <c r="D69" s="12" t="inlineStr">
         <is>
-          <t>BIBS_CR_BRD-02_Remittance_Effort_Estimate_v1.0</t>
+          <t>BIBS_USR-BDOI_BRD-02_Operations_Cashiering_User_Stories_v1.0</t>
         </is>
       </c>
       <c r="E69" s="12" t="inlineStr">
@@ -4507,7 +4507,7 @@
       </c>
       <c r="G69" s="12" t="inlineStr">
         <is>
-          <t>17 Oct 2026</t>
+          <t>16 Oct 2026</t>
         </is>
       </c>
       <c r="H69" s="12" t="inlineStr">
@@ -4534,32 +4534,32 @@
       </c>
       <c r="B70" s="12" t="inlineStr">
         <is>
-          <t>DDI</t>
+          <t>UXD</t>
         </is>
       </c>
       <c r="C70" s="12" t="inlineStr">
         <is>
-          <t>Operations Remittance Data Dictionary</t>
+          <t>Operations Cashiering UX Design</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
         <is>
-          <t>BIBS_DDI-BDOI_BRD-02_Operations_Remittance_Data_Dictionary_v1.1</t>
+          <t>BIBS_UXD-BDOI_BRD-02_Operations_Cashiering_UX_Design_v3.4</t>
         </is>
       </c>
       <c r="E70" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F70" s="12" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="G70" s="12" t="inlineStr">
         <is>
-          <t>17 Oct 2026</t>
+          <t>16 Oct 2026</t>
         </is>
       </c>
       <c r="H70" s="12" t="inlineStr">
@@ -4586,27 +4586,27 @@
       </c>
       <c r="B71" s="12" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>Access</t>
         </is>
       </c>
       <c r="C71" s="12" t="inlineStr">
         <is>
-          <t>Operations Remittance Developer Specification</t>
+          <t>Remittance Access Matrix</t>
         </is>
       </c>
       <c r="D71" s="12" t="inlineStr">
         <is>
-          <t>BIBS_DSP-BDOI_BRD-02_Operations_Remittance_Developer_Specification_v1.1</t>
+          <t>BIBS_Access_BRD-02_Remittance_Access_Matrix_v1.0</t>
         </is>
       </c>
       <c r="E71" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F71" s="12" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G71" s="12" t="inlineStr">
@@ -4638,17 +4638,17 @@
       </c>
       <c r="B72" s="12" t="inlineStr">
         <is>
-          <t>FRS</t>
+          <t>BPS</t>
         </is>
       </c>
       <c r="C72" s="12" t="inlineStr">
         <is>
-          <t>Operations Remittance</t>
+          <t>Operations Remittance Process and Storyboards</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FRS-BDOI_BRD-02_Operations_Remittance_v1.0</t>
+          <t>BIBS_BPS-BDOI_BRD-02_Operations_Remittance_Process_and_Storyboards_v1.0</t>
         </is>
       </c>
       <c r="E72" s="12" t="inlineStr">
@@ -4690,17 +4690,17 @@
       </c>
       <c r="B73" s="12" t="inlineStr">
         <is>
-          <t>FitGap</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C73" s="12" t="inlineStr">
         <is>
-          <t>Remittance BRD vs OOTB vs Best Practice</t>
+          <t>Remittance Change Request Register</t>
         </is>
       </c>
       <c r="D73" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FitGap_BRD-02_Remittance_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+          <t>BIBS_CR_BRD-02_Remittance_Change_Request_Register_v1.0</t>
         </is>
       </c>
       <c r="E73" s="12" t="inlineStr">
@@ -4742,22 +4742,22 @@
       </c>
       <c r="B74" s="12" t="inlineStr">
         <is>
-          <t>ICD</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C74" s="12" t="inlineStr">
         <is>
-          <t>Operations Remittance Interface Specification</t>
+          <t>Remittance Effort Estimate</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
         <is>
-          <t>BIBS_ICD-BDOI_BRD-02_Operations_Remittance_Interface_Specification_v1.0</t>
+          <t>BIBS_CR_BRD-02_Remittance_Effort_Estimate_v1.0</t>
         </is>
       </c>
       <c r="E74" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F74" s="12" t="inlineStr">
@@ -4794,17 +4794,17 @@
       </c>
       <c r="B75" s="12" t="inlineStr">
         <is>
-          <t>Inputs</t>
+          <t>DDI</t>
         </is>
       </c>
       <c r="C75" s="12" t="inlineStr">
         <is>
-          <t>Remittance Business Unit Requirements Collection</t>
+          <t>Operations Remittance Data Dictionary</t>
         </is>
       </c>
       <c r="D75" s="12" t="inlineStr">
         <is>
-          <t>BIBS_Inputs_BRD-02_Remittance_Business_Unit_Requirements_Collection_v1.0</t>
+          <t>BIBS_DDI-BDOI_BRD-02_Operations_Remittance_Data_Dictionary_v1.1</t>
         </is>
       </c>
       <c r="E75" s="12" t="inlineStr">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="F75" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G75" s="12" t="inlineStr">
@@ -4846,17 +4846,17 @@
       </c>
       <c r="B76" s="12" t="inlineStr">
         <is>
-          <t>README</t>
+          <t>DSP</t>
         </is>
       </c>
       <c r="C76" s="12" t="inlineStr">
         <is>
-          <t>Remittance How to Read this Pack</t>
+          <t>Operations Remittance Developer Specification</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
         <is>
-          <t>BIBS_Inputs_BRD-02_Remittance_How_to_Read_this_Pack_v1.0</t>
+          <t>BIBS_DSP-BDOI_BRD-02_Operations_Remittance_Developer_Specification_v1.1</t>
         </is>
       </c>
       <c r="E76" s="12" t="inlineStr">
@@ -4866,7 +4866,7 @@
       </c>
       <c r="F76" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G76" s="12" t="inlineStr">
@@ -4898,17 +4898,17 @@
       </c>
       <c r="B77" s="12" t="inlineStr">
         <is>
-          <t>RNO</t>
+          <t>FRS</t>
         </is>
       </c>
       <c r="C77" s="12" t="inlineStr">
         <is>
-          <t>Operations Remittance Reports Notifications Outputs</t>
+          <t>Operations Remittance</t>
         </is>
       </c>
       <c r="D77" s="12" t="inlineStr">
         <is>
-          <t>BIBS_RNO-BDOI_BRD-02_Operations_Remittance_Reports_Notifications_Outputs_v1.1</t>
+          <t>BIBS_FRS-BDOI_BRD-02_Operations_Remittance_v1.0</t>
         </is>
       </c>
       <c r="E77" s="12" t="inlineStr">
@@ -4918,7 +4918,7 @@
       </c>
       <c r="F77" s="12" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G77" s="12" t="inlineStr">
@@ -4950,17 +4950,17 @@
       </c>
       <c r="B78" s="12" t="inlineStr">
         <is>
-          <t>RTM</t>
+          <t>FitGap</t>
         </is>
       </c>
       <c r="C78" s="12" t="inlineStr">
         <is>
-          <t>Remittance Test Cases and Traceability</t>
+          <t>Remittance BRD vs OOTB vs Best Practice</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
         <is>
-          <t>BIBS_RTM_BRD-02_Remittance_Test_Cases_and_Traceability_v1.0</t>
+          <t>BIBS_FitGap_BRD-02_Remittance_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
         </is>
       </c>
       <c r="E78" s="12" t="inlineStr">
@@ -5002,22 +5002,22 @@
       </c>
       <c r="B79" s="12" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>ICD</t>
         </is>
       </c>
       <c r="C79" s="12" t="inlineStr">
         <is>
-          <t>Remittance Business Unit Walkthrough Users</t>
+          <t>Operations Remittance Interface Specification</t>
         </is>
       </c>
       <c r="D79" s="12" t="inlineStr">
         <is>
-          <t>BIBS_UAT_BRD-02_Remittance_Business_Unit_Walkthrough_Users_v1.0</t>
+          <t>BIBS_ICD-BDOI_BRD-02_Operations_Remittance_Interface_Specification_v1.0</t>
         </is>
       </c>
       <c r="E79" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F79" s="12" t="inlineStr">
@@ -5054,17 +5054,17 @@
       </c>
       <c r="B80" s="12" t="inlineStr">
         <is>
-          <t>USR</t>
+          <t>Inputs</t>
         </is>
       </c>
       <c r="C80" s="12" t="inlineStr">
         <is>
-          <t>Operations Remittance User Stories</t>
+          <t>Remittance Business Unit Requirements Collection</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
         <is>
-          <t>BIBS_USR-BDOI_BRD-02_Operations_Remittance_User_Stories_v1.0</t>
+          <t>BIBS_Inputs_BRD-02_Remittance_Business_Unit_Requirements_Collection_v1.0</t>
         </is>
       </c>
       <c r="E80" s="12" t="inlineStr">
@@ -5106,17 +5106,17 @@
       </c>
       <c r="B81" s="12" t="inlineStr">
         <is>
-          <t>UXD</t>
+          <t>README</t>
         </is>
       </c>
       <c r="C81" s="12" t="inlineStr">
         <is>
-          <t>Operations Remittance UX Design</t>
+          <t>Remittance How to Read this Pack</t>
         </is>
       </c>
       <c r="D81" s="12" t="inlineStr">
         <is>
-          <t>BIBS_UXD-BDOI_BRD-02_Operations_Remittance_UX_Design_v1.1</t>
+          <t>BIBS_Inputs_BRD-02_Remittance_How_to_Read_this_Pack_v1.0</t>
         </is>
       </c>
       <c r="E81" s="12" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="F81" s="12" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G81" s="12" t="inlineStr">
@@ -5153,22 +5153,22 @@
     <row r="82">
       <c r="A82" s="12" t="inlineStr">
         <is>
-          <t>BRD-07</t>
+          <t>BRD-02</t>
         </is>
       </c>
       <c r="B82" s="12" t="inlineStr">
         <is>
-          <t>BPS</t>
+          <t>RNO</t>
         </is>
       </c>
       <c r="C82" s="12" t="inlineStr">
         <is>
-          <t>Claims Process and Storyboards</t>
+          <t>Operations Remittance Reports Notifications Outputs</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
         <is>
-          <t>BIBS_BPS-BDOI_BRD-07_Claims_Process_and_Storyboards_v1.0</t>
+          <t>BIBS_RNO-BDOI_BRD-02_Operations_Remittance_Reports_Notifications_Outputs_v1.1</t>
         </is>
       </c>
       <c r="E82" s="12" t="inlineStr">
@@ -5178,7 +5178,7 @@
       </c>
       <c r="F82" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G82" s="12" t="inlineStr">
@@ -5188,7 +5188,7 @@
       </c>
       <c r="H82" s="12" t="inlineStr">
         <is>
-          <t>BDOI Product Owner, Claims</t>
+          <t>BDOI Product Owner, Operations</t>
         </is>
       </c>
       <c r="I82" s="12" t="inlineStr">
@@ -5205,22 +5205,22 @@
     <row r="83">
       <c r="A83" s="12" t="inlineStr">
         <is>
-          <t>BRD-07</t>
+          <t>BRD-02</t>
         </is>
       </c>
       <c r="B83" s="12" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>RTM</t>
         </is>
       </c>
       <c r="C83" s="12" t="inlineStr">
         <is>
-          <t>Claims Change Request Register</t>
+          <t>Remittance Test Cases and Traceability</t>
         </is>
       </c>
       <c r="D83" s="12" t="inlineStr">
         <is>
-          <t>BIBS_CR_BRD-07_Claims_Change_Request_Register_v1.0</t>
+          <t>BIBS_RTM_BRD-02_Remittance_Test_Cases_and_Traceability_v1.0</t>
         </is>
       </c>
       <c r="E83" s="12" t="inlineStr">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="H83" s="12" t="inlineStr">
         <is>
-          <t>BDOI Product Owner, Claims</t>
+          <t>BDOI Product Owner, Operations</t>
         </is>
       </c>
       <c r="I83" s="12" t="inlineStr">
@@ -5257,22 +5257,22 @@
     <row r="84">
       <c r="A84" s="12" t="inlineStr">
         <is>
-          <t>BRD-07</t>
+          <t>BRD-02</t>
         </is>
       </c>
       <c r="B84" s="12" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="C84" s="12" t="inlineStr">
         <is>
-          <t>Claims Effort Estimate</t>
+          <t>Remittance Business Unit Walkthrough Users</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
         <is>
-          <t>BIBS_CR_BRD-07_Claims_Effort_Estimate_v1.0</t>
+          <t>BIBS_UAT_BRD-02_Remittance_Business_Unit_Walkthrough_Users_v1.0</t>
         </is>
       </c>
       <c r="E84" s="12" t="inlineStr">
@@ -5292,7 +5292,7 @@
       </c>
       <c r="H84" s="12" t="inlineStr">
         <is>
-          <t>BDOI Product Owner, Claims</t>
+          <t>BDOI Product Owner, Operations</t>
         </is>
       </c>
       <c r="I84" s="12" t="inlineStr">
@@ -5309,22 +5309,22 @@
     <row r="85">
       <c r="A85" s="12" t="inlineStr">
         <is>
-          <t>BRD-07</t>
+          <t>BRD-02</t>
         </is>
       </c>
       <c r="B85" s="12" t="inlineStr">
         <is>
-          <t>DDI</t>
+          <t>USR</t>
         </is>
       </c>
       <c r="C85" s="12" t="inlineStr">
         <is>
-          <t>Claims Data Dictionary</t>
+          <t>Operations Remittance User Stories</t>
         </is>
       </c>
       <c r="D85" s="12" t="inlineStr">
         <is>
-          <t>BIBS_DDI-BDOI_BRD-07_Claims_Data_Dictionary_v1.1</t>
+          <t>BIBS_USR-BDOI_BRD-02_Operations_Remittance_User_Stories_v1.0</t>
         </is>
       </c>
       <c r="E85" s="12" t="inlineStr">
@@ -5334,7 +5334,7 @@
       </c>
       <c r="F85" s="12" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G85" s="12" t="inlineStr">
@@ -5344,7 +5344,7 @@
       </c>
       <c r="H85" s="12" t="inlineStr">
         <is>
-          <t>BDOI Product Owner, Claims</t>
+          <t>BDOI Product Owner, Operations</t>
         </is>
       </c>
       <c r="I85" s="12" t="inlineStr">
@@ -5361,22 +5361,22 @@
     <row r="86">
       <c r="A86" s="12" t="inlineStr">
         <is>
-          <t>BRD-07</t>
+          <t>BRD-02</t>
         </is>
       </c>
       <c r="B86" s="12" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>UXD</t>
         </is>
       </c>
       <c r="C86" s="12" t="inlineStr">
         <is>
-          <t>Claims Developer Specification</t>
+          <t>Operations Remittance UX Design</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
         <is>
-          <t>BIBS_DSP-BDOI_BRD-07_Claims_Developer_Specification_v1.1</t>
+          <t>BIBS_UXD-BDOI_BRD-02_Operations_Remittance_UX_Design_v1.1</t>
         </is>
       </c>
       <c r="E86" s="12" t="inlineStr">
@@ -5396,7 +5396,7 @@
       </c>
       <c r="H86" s="12" t="inlineStr">
         <is>
-          <t>BDOI Product Owner, Claims</t>
+          <t>BDOI Product Owner, Operations</t>
         </is>
       </c>
       <c r="I86" s="12" t="inlineStr">
@@ -5418,22 +5418,22 @@
       </c>
       <c r="B87" s="12" t="inlineStr">
         <is>
-          <t>FRS</t>
+          <t>Access</t>
         </is>
       </c>
       <c r="C87" s="12" t="inlineStr">
         <is>
-          <t>Claims</t>
+          <t>Claims Access Matrix</t>
         </is>
       </c>
       <c r="D87" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FRS-BDOI_BRD-07_Claims_v1.0</t>
+          <t>BIBS_Access_BRD-07_Claims_Access_Matrix_v1.0</t>
         </is>
       </c>
       <c r="E87" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F87" s="12" t="inlineStr">
@@ -5470,22 +5470,22 @@
       </c>
       <c r="B88" s="12" t="inlineStr">
         <is>
-          <t>FitGap</t>
+          <t>BPS</t>
         </is>
       </c>
       <c r="C88" s="12" t="inlineStr">
         <is>
-          <t>Claims BRD vs OOTB vs Best Practice</t>
+          <t>Claims Process and Storyboards</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FitGap_BRD-07_Claims_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+          <t>BIBS_BPS-BDOI_BRD-07_Claims_Process_and_Storyboards_v1.0</t>
         </is>
       </c>
       <c r="E88" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F88" s="12" t="inlineStr">
@@ -5522,22 +5522,22 @@
       </c>
       <c r="B89" s="12" t="inlineStr">
         <is>
-          <t>ICD</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C89" s="12" t="inlineStr">
         <is>
-          <t>Claims Interface Specification</t>
+          <t>Claims Change Request Register</t>
         </is>
       </c>
       <c r="D89" s="12" t="inlineStr">
         <is>
-          <t>BIBS_ICD-BDOI_BRD-07_Claims_Interface_Specification_v1.0</t>
+          <t>BIBS_CR_BRD-07_Claims_Change_Request_Register_v1.0</t>
         </is>
       </c>
       <c r="E89" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F89" s="12" t="inlineStr">
@@ -5574,17 +5574,17 @@
       </c>
       <c r="B90" s="12" t="inlineStr">
         <is>
-          <t>Inputs</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C90" s="12" t="inlineStr">
         <is>
-          <t>Claims Business Unit Requirements Collection</t>
+          <t>Claims Effort Estimate</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr">
         <is>
-          <t>BIBS_Inputs_BRD-07_Claims_Business_Unit_Requirements_Collection_v1.0</t>
+          <t>BIBS_CR_BRD-07_Claims_Effort_Estimate_v1.0</t>
         </is>
       </c>
       <c r="E90" s="12" t="inlineStr">
@@ -5626,27 +5626,27 @@
       </c>
       <c r="B91" s="12" t="inlineStr">
         <is>
-          <t>README</t>
+          <t>DDI</t>
         </is>
       </c>
       <c r="C91" s="12" t="inlineStr">
         <is>
-          <t>Claims How to Read this Pack</t>
+          <t>Claims Data Dictionary</t>
         </is>
       </c>
       <c r="D91" s="12" t="inlineStr">
         <is>
-          <t>BIBS_Inputs_BRD-07_Claims_How_to_Read_this_Pack_v1.0</t>
+          <t>BIBS_DDI-BDOI_BRD-07_Claims_Data_Dictionary_v1.1</t>
         </is>
       </c>
       <c r="E91" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F91" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G91" s="12" t="inlineStr">
@@ -5678,17 +5678,17 @@
       </c>
       <c r="B92" s="12" t="inlineStr">
         <is>
-          <t>RNO</t>
+          <t>DSP</t>
         </is>
       </c>
       <c r="C92" s="12" t="inlineStr">
         <is>
-          <t>Claims Reports Notifications Outputs</t>
+          <t>Claims Developer Specification</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr">
         <is>
-          <t>BIBS_RNO-BDOI_BRD-07_Claims_Reports_Notifications_Outputs_v1.1</t>
+          <t>BIBS_DSP-BDOI_BRD-07_Claims_Developer_Specification_v1.1</t>
         </is>
       </c>
       <c r="E92" s="12" t="inlineStr">
@@ -5730,22 +5730,22 @@
       </c>
       <c r="B93" s="12" t="inlineStr">
         <is>
-          <t>RTM</t>
+          <t>FRS</t>
         </is>
       </c>
       <c r="C93" s="12" t="inlineStr">
         <is>
-          <t>Claims Test Cases and Traceability</t>
+          <t>Claims</t>
         </is>
       </c>
       <c r="D93" s="12" t="inlineStr">
         <is>
-          <t>BIBS_RTM_BRD-07_Claims_Test_Cases_and_Traceability_v1.0</t>
+          <t>BIBS_FRS-BDOI_BRD-07_Claims_v1.0</t>
         </is>
       </c>
       <c r="E93" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F93" s="12" t="inlineStr">
@@ -5782,17 +5782,17 @@
       </c>
       <c r="B94" s="12" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>FitGap</t>
         </is>
       </c>
       <c r="C94" s="12" t="inlineStr">
         <is>
-          <t>Claims Business Unit Walkthrough Users</t>
+          <t>Claims BRD vs OOTB vs Best Practice</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
         <is>
-          <t>BIBS_UAT_BRD-07_Claims_Business_Unit_Walkthrough_Users_v1.0</t>
+          <t>BIBS_FitGap_BRD-07_Claims_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
         </is>
       </c>
       <c r="E94" s="12" t="inlineStr">
@@ -5834,22 +5834,22 @@
       </c>
       <c r="B95" s="12" t="inlineStr">
         <is>
-          <t>USR</t>
+          <t>ICD</t>
         </is>
       </c>
       <c r="C95" s="12" t="inlineStr">
         <is>
-          <t>Claims User Stories</t>
+          <t>Claims Interface Specification</t>
         </is>
       </c>
       <c r="D95" s="12" t="inlineStr">
         <is>
-          <t>BIBS_USR-BDOI_BRD-07_Claims_User_Stories_v1.0</t>
+          <t>BIBS_ICD-BDOI_BRD-07_Claims_Interface_Specification_v1.0</t>
         </is>
       </c>
       <c r="E95" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F95" s="12" t="inlineStr">
@@ -5886,27 +5886,27 @@
       </c>
       <c r="B96" s="12" t="inlineStr">
         <is>
-          <t>UXD</t>
+          <t>Inputs</t>
         </is>
       </c>
       <c r="C96" s="12" t="inlineStr">
         <is>
-          <t>Claims UX Design</t>
+          <t>Claims Business Unit Requirements Collection</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
         <is>
-          <t>BIBS_UXD-BDOI_BRD-07_Claims_UX_Design_v1.1</t>
+          <t>BIBS_Inputs_BRD-07_Claims_Business_Unit_Requirements_Collection_v1.0</t>
         </is>
       </c>
       <c r="E96" s="12" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="F96" s="12" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G96" s="12" t="inlineStr">
@@ -5933,22 +5933,22 @@
     <row r="97">
       <c r="A97" s="12" t="inlineStr">
         <is>
-          <t>Programme</t>
+          <t>BRD-07</t>
         </is>
       </c>
       <c r="B97" s="12" t="inlineStr">
         <is>
-          <t>NFR</t>
+          <t>README</t>
         </is>
       </c>
       <c r="C97" s="12" t="inlineStr">
         <is>
-          <t>Non Functional and Security Requirements</t>
+          <t>Claims How to Read this Pack</t>
         </is>
       </c>
       <c r="D97" s="12" t="inlineStr">
         <is>
-          <t>BIBS_NFR_BRD-00_Non_Functional_and_Security_Requirements_v2.0</t>
+          <t>BIBS_Inputs_BRD-07_Claims_How_to_Read_this_Pack_v1.0</t>
         </is>
       </c>
       <c r="E97" s="12" t="inlineStr">
@@ -5958,17 +5958,17 @@
       </c>
       <c r="F97" s="12" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G97" s="12" t="inlineStr">
         <is>
-          <t>16 Oct 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="H97" s="12" t="inlineStr">
         <is>
-          <t>BIBS Product Owner</t>
+          <t>BDOI Product Owner, Claims</t>
         </is>
       </c>
       <c r="I97" s="12" t="inlineStr">
@@ -5985,42 +5985,42 @@
     <row r="98">
       <c r="A98" s="12" t="inlineStr">
         <is>
-          <t>Programme</t>
+          <t>BRD-07</t>
         </is>
       </c>
       <c r="B98" s="12" t="inlineStr">
         <is>
-          <t>Glossary</t>
+          <t>RNO</t>
         </is>
       </c>
       <c r="C98" s="12" t="inlineStr">
         <is>
-          <t>Programme Glossary</t>
+          <t>Claims Reports Notifications Outputs</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
         <is>
-          <t>BIBS_Glossary_BRD-00_Programme_Glossary_v1.0</t>
+          <t>BIBS_RNO-BDOI_BRD-07_Claims_Reports_Notifications_Outputs_v1.1</t>
         </is>
       </c>
       <c r="E98" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F98" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G98" s="12" t="inlineStr">
         <is>
-          <t>16 Oct 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="H98" s="12" t="inlineStr">
         <is>
-          <t>BIBS Product Owner</t>
+          <t>BDOI Product Owner, Claims</t>
         </is>
       </c>
       <c r="I98" s="12" t="inlineStr">
@@ -6037,22 +6037,22 @@
     <row r="99">
       <c r="A99" s="12" t="inlineStr">
         <is>
-          <t>Programme</t>
+          <t>BRD-07</t>
         </is>
       </c>
       <c r="B99" s="12" t="inlineStr">
         <is>
-          <t>Log</t>
+          <t>RTM</t>
         </is>
       </c>
       <c r="C99" s="12" t="inlineStr">
         <is>
-          <t>Decision and Observation Log</t>
+          <t>Claims Test Cases and Traceability</t>
         </is>
       </c>
       <c r="D99" s="12" t="inlineStr">
         <is>
-          <t>BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0</t>
+          <t>BIBS_RTM_BRD-07_Claims_Test_Cases_and_Traceability_v1.0</t>
         </is>
       </c>
       <c r="E99" s="12" t="inlineStr">
@@ -6067,12 +6067,12 @@
       </c>
       <c r="G99" s="12" t="inlineStr">
         <is>
-          <t>16 Oct 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="H99" s="12" t="inlineStr">
         <is>
-          <t>BIBS Product Owner</t>
+          <t>BDOI Product Owner, Claims</t>
         </is>
       </c>
       <c r="I99" s="12" t="inlineStr">
@@ -6089,22 +6089,22 @@
     <row r="100">
       <c r="A100" s="12" t="inlineStr">
         <is>
-          <t>BRD-00</t>
+          <t>BRD-07</t>
         </is>
       </c>
       <c r="B100" s="12" t="inlineStr">
         <is>
-          <t>FitGap</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="C100" s="12" t="inlineStr">
         <is>
-          <t>Core Replacement BRD vs OOTB vs Best Practice</t>
+          <t>Claims Business Unit Walkthrough Users</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FitGap_BRD-00_Core_Replacement_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+          <t>BIBS_UAT_BRD-07_Claims_Business_Unit_Walkthrough_Users_v1.0</t>
         </is>
       </c>
       <c r="E100" s="12" t="inlineStr">
@@ -6119,12 +6119,12 @@
       </c>
       <c r="G100" s="12" t="inlineStr">
         <is>
-          <t>16 Oct 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="H100" s="12" t="inlineStr">
         <is>
-          <t>BIBS Product Owner</t>
+          <t>BDOI Product Owner, Claims</t>
         </is>
       </c>
       <c r="I100" s="12" t="inlineStr">
@@ -6141,22 +6141,22 @@
     <row r="101">
       <c r="A101" s="12" t="inlineStr">
         <is>
-          <t>BRD-00</t>
+          <t>BRD-07</t>
         </is>
       </c>
       <c r="B101" s="12" t="inlineStr">
         <is>
-          <t>FitGap</t>
+          <t>USR</t>
         </is>
       </c>
       <c r="C101" s="12" t="inlineStr">
         <is>
-          <t>Summary All BRDs</t>
+          <t>Claims User Stories</t>
         </is>
       </c>
       <c r="D101" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FitGap_BRD-00_Summary_All_BRDs_v1.0</t>
+          <t>BIBS_USR-BDOI_BRD-07_Claims_User_Stories_v1.0</t>
         </is>
       </c>
       <c r="E101" s="12" t="inlineStr">
@@ -6171,12 +6171,12 @@
       </c>
       <c r="G101" s="12" t="inlineStr">
         <is>
-          <t>16 Oct 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="H101" s="12" t="inlineStr">
         <is>
-          <t>BIBS Product Owner</t>
+          <t>BDOI Product Owner, Claims</t>
         </is>
       </c>
       <c r="I101" s="12" t="inlineStr">
@@ -6193,42 +6193,42 @@
     <row r="102">
       <c r="A102" s="12" t="inlineStr">
         <is>
-          <t>BRD-01</t>
+          <t>BRD-07</t>
         </is>
       </c>
       <c r="B102" s="12" t="inlineStr">
         <is>
-          <t>FitGap</t>
+          <t>UXD</t>
         </is>
       </c>
       <c r="C102" s="12" t="inlineStr">
         <is>
-          <t>New Business BRD vs OOTB vs Best Practice</t>
+          <t>Claims UX Design</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FitGap_BRD-01_New_Business_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+          <t>BIBS_UXD-BDOI_BRD-07_Claims_UX_Design_v1.1</t>
         </is>
       </c>
       <c r="E102" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F102" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G102" s="12" t="inlineStr">
         <is>
-          <t>16 Oct 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="H102" s="12" t="inlineStr">
         <is>
-          <t>BIBS Product Owner</t>
+          <t>BDOI Product Owner, Claims</t>
         </is>
       </c>
       <c r="I102" s="12" t="inlineStr">
@@ -6245,32 +6245,32 @@
     <row r="103">
       <c r="A103" s="12" t="inlineStr">
         <is>
-          <t>BRD-04</t>
+          <t>Programme</t>
         </is>
       </c>
       <c r="B103" s="12" t="inlineStr">
         <is>
-          <t>FitGap</t>
+          <t>NFR</t>
         </is>
       </c>
       <c r="C103" s="12" t="inlineStr">
         <is>
-          <t>Collections BRD vs OOTB vs Best Practice</t>
+          <t>Non Functional and Security Requirements</t>
         </is>
       </c>
       <c r="D103" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FitGap_BRD-04_Collections_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+          <t>BIBS_NFR_BRD-00_Non_Functional_and_Security_Requirements_v2.0</t>
         </is>
       </c>
       <c r="E103" s="12" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>DOCX</t>
         </is>
       </c>
       <c r="F103" s="12" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="G103" s="12" t="inlineStr">
@@ -6297,22 +6297,22 @@
     <row r="104">
       <c r="A104" s="12" t="inlineStr">
         <is>
-          <t>BRD-05</t>
+          <t>Programme</t>
         </is>
       </c>
       <c r="B104" s="12" t="inlineStr">
         <is>
-          <t>FitGap</t>
+          <t>Glossary</t>
         </is>
       </c>
       <c r="C104" s="12" t="inlineStr">
         <is>
-          <t>Accounting Disbursement ACSL BRD vs OOTB vs Best Practice</t>
+          <t>Programme Glossary</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FitGap_BRD-05_Accounting_Disbursement_ACSL_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+          <t>BIBS_Glossary_BRD-00_Programme_Glossary_v1.0</t>
         </is>
       </c>
       <c r="E104" s="12" t="inlineStr">
@@ -6349,22 +6349,22 @@
     <row r="105">
       <c r="A105" s="12" t="inlineStr">
         <is>
-          <t>BRD-07</t>
+          <t>Programme</t>
         </is>
       </c>
       <c r="B105" s="12" t="inlineStr">
         <is>
-          <t>FitGap</t>
+          <t>Log</t>
         </is>
       </c>
       <c r="C105" s="12" t="inlineStr">
         <is>
-          <t>Claims BRD vs OOTB vs Best Practice</t>
+          <t>Decision and Observation Log</t>
         </is>
       </c>
       <c r="D105" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FitGap_BRD-07_Claims_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+          <t>BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0</t>
         </is>
       </c>
       <c r="E105" s="12" t="inlineStr">
@@ -6401,7 +6401,7 @@
     <row r="106">
       <c r="A106" s="12" t="inlineStr">
         <is>
-          <t>BRD-08</t>
+          <t>BRD-00</t>
         </is>
       </c>
       <c r="B106" s="12" t="inlineStr">
@@ -6411,12 +6411,12 @@
       </c>
       <c r="C106" s="12" t="inlineStr">
         <is>
-          <t>Employee Benefits BRD vs OOTB vs Best Practice</t>
+          <t>Core Replacement BRD vs OOTB vs Best Practice</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FitGap_BRD-08_Employee_Benefits_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+          <t>BIBS_FitGap_BRD-00_Core_Replacement_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
         </is>
       </c>
       <c r="E106" s="12" t="inlineStr">
@@ -6453,7 +6453,7 @@
     <row r="107">
       <c r="A107" s="12" t="inlineStr">
         <is>
-          <t>BRD-09</t>
+          <t>BRD-00</t>
         </is>
       </c>
       <c r="B107" s="12" t="inlineStr">
@@ -6463,12 +6463,12 @@
       </c>
       <c r="C107" s="12" t="inlineStr">
         <is>
-          <t>Customer Servicing Facility BRD vs OOTB vs Best Practice</t>
+          <t>Summary All BRDs</t>
         </is>
       </c>
       <c r="D107" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FitGap_BRD-09_Customer_Servicing_Facility_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+          <t>BIBS_FitGap_BRD-00_Summary_All_BRDs_v1.0</t>
         </is>
       </c>
       <c r="E107" s="12" t="inlineStr">
@@ -6505,7 +6505,7 @@
     <row r="108">
       <c r="A108" s="12" t="inlineStr">
         <is>
-          <t>BRD-10</t>
+          <t>BRD-01</t>
         </is>
       </c>
       <c r="B108" s="12" t="inlineStr">
@@ -6515,12 +6515,12 @@
       </c>
       <c r="C108" s="12" t="inlineStr">
         <is>
-          <t>Sanction Screening BRD vs OOTB vs Best Practice</t>
+          <t>New Business BRD vs OOTB vs Best Practice</t>
         </is>
       </c>
       <c r="D108" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FitGap_BRD-10_Sanction_Screening_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+          <t>BIBS_FitGap_BRD-01_New_Business_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
         </is>
       </c>
       <c r="E108" s="12" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="109">
       <c r="A109" s="12" t="inlineStr">
         <is>
-          <t>BRD-12</t>
+          <t>BRD-04</t>
         </is>
       </c>
       <c r="B109" s="12" t="inlineStr">
@@ -6567,12 +6567,12 @@
       </c>
       <c r="C109" s="12" t="inlineStr">
         <is>
-          <t>Submitted Policies BRD vs OOTB vs Best Practice</t>
+          <t>Collections BRD vs OOTB vs Best Practice</t>
         </is>
       </c>
       <c r="D109" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FitGap_BRD-12_Submitted_Policies_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+          <t>BIBS_FitGap_BRD-04_Collections_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
         </is>
       </c>
       <c r="E109" s="12" t="inlineStr">
@@ -6609,7 +6609,7 @@
     <row r="110">
       <c r="A110" s="12" t="inlineStr">
         <is>
-          <t>BRD-13</t>
+          <t>BRD-05</t>
         </is>
       </c>
       <c r="B110" s="12" t="inlineStr">
@@ -6619,12 +6619,12 @@
       </c>
       <c r="C110" s="12" t="inlineStr">
         <is>
-          <t>Data Migration BRD vs OOTB vs Best Practice</t>
+          <t>Accounting Disbursement ACSL BRD vs OOTB vs Best Practice</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
         <is>
-          <t>BIBS_FitGap_BRD-13_Data_Migration_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+          <t>BIBS_FitGap_BRD-05_Accounting_Disbursement_ACSL_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
         </is>
       </c>
       <c r="E110" s="12" t="inlineStr">
@@ -6661,67 +6661,379 @@
     <row r="111">
       <c r="A111" s="12" t="inlineStr">
         <is>
+          <t>BRD-07</t>
+        </is>
+      </c>
+      <c r="B111" s="12" t="inlineStr">
+        <is>
+          <t>FitGap</t>
+        </is>
+      </c>
+      <c r="C111" s="12" t="inlineStr">
+        <is>
+          <t>Claims BRD vs OOTB vs Best Practice</t>
+        </is>
+      </c>
+      <c r="D111" s="12" t="inlineStr">
+        <is>
+          <t>BIBS_FitGap_BRD-07_Claims_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+        </is>
+      </c>
+      <c r="E111" s="12" t="inlineStr">
+        <is>
+          <t>XLSX</t>
+        </is>
+      </c>
+      <c r="F111" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G111" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H111" s="12" t="inlineStr">
+        <is>
+          <t>BIBS Product Owner</t>
+        </is>
+      </c>
+      <c r="I111" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="J111" s="22" t="inlineStr">
+        <is>
+          <t>Issued for BDOI review</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="12" t="inlineStr">
+        <is>
+          <t>BRD-08</t>
+        </is>
+      </c>
+      <c r="B112" s="12" t="inlineStr">
+        <is>
+          <t>FitGap</t>
+        </is>
+      </c>
+      <c r="C112" s="12" t="inlineStr">
+        <is>
+          <t>Employee Benefits BRD vs OOTB vs Best Practice</t>
+        </is>
+      </c>
+      <c r="D112" s="12" t="inlineStr">
+        <is>
+          <t>BIBS_FitGap_BRD-08_Employee_Benefits_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+        </is>
+      </c>
+      <c r="E112" s="12" t="inlineStr">
+        <is>
+          <t>XLSX</t>
+        </is>
+      </c>
+      <c r="F112" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G112" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H112" s="12" t="inlineStr">
+        <is>
+          <t>BIBS Product Owner</t>
+        </is>
+      </c>
+      <c r="I112" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="J112" s="22" t="inlineStr">
+        <is>
+          <t>Issued for BDOI review</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="12" t="inlineStr">
+        <is>
+          <t>BRD-09</t>
+        </is>
+      </c>
+      <c r="B113" s="12" t="inlineStr">
+        <is>
+          <t>FitGap</t>
+        </is>
+      </c>
+      <c r="C113" s="12" t="inlineStr">
+        <is>
+          <t>Customer Servicing Facility BRD vs OOTB vs Best Practice</t>
+        </is>
+      </c>
+      <c r="D113" s="12" t="inlineStr">
+        <is>
+          <t>BIBS_FitGap_BRD-09_Customer_Servicing_Facility_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+        </is>
+      </c>
+      <c r="E113" s="12" t="inlineStr">
+        <is>
+          <t>XLSX</t>
+        </is>
+      </c>
+      <c r="F113" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G113" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H113" s="12" t="inlineStr">
+        <is>
+          <t>BIBS Product Owner</t>
+        </is>
+      </c>
+      <c r="I113" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="J113" s="22" t="inlineStr">
+        <is>
+          <t>Issued for BDOI review</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="12" t="inlineStr">
+        <is>
+          <t>BRD-10</t>
+        </is>
+      </c>
+      <c r="B114" s="12" t="inlineStr">
+        <is>
+          <t>FitGap</t>
+        </is>
+      </c>
+      <c r="C114" s="12" t="inlineStr">
+        <is>
+          <t>Sanction Screening BRD vs OOTB vs Best Practice</t>
+        </is>
+      </c>
+      <c r="D114" s="12" t="inlineStr">
+        <is>
+          <t>BIBS_FitGap_BRD-10_Sanction_Screening_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+        </is>
+      </c>
+      <c r="E114" s="12" t="inlineStr">
+        <is>
+          <t>XLSX</t>
+        </is>
+      </c>
+      <c r="F114" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G114" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H114" s="12" t="inlineStr">
+        <is>
+          <t>BIBS Product Owner</t>
+        </is>
+      </c>
+      <c r="I114" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="J114" s="22" t="inlineStr">
+        <is>
+          <t>Issued for BDOI review</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="12" t="inlineStr">
+        <is>
+          <t>BRD-12</t>
+        </is>
+      </c>
+      <c r="B115" s="12" t="inlineStr">
+        <is>
+          <t>FitGap</t>
+        </is>
+      </c>
+      <c r="C115" s="12" t="inlineStr">
+        <is>
+          <t>Submitted Policies BRD vs OOTB vs Best Practice</t>
+        </is>
+      </c>
+      <c r="D115" s="12" t="inlineStr">
+        <is>
+          <t>BIBS_FitGap_BRD-12_Submitted_Policies_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+        </is>
+      </c>
+      <c r="E115" s="12" t="inlineStr">
+        <is>
+          <t>XLSX</t>
+        </is>
+      </c>
+      <c r="F115" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G115" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H115" s="12" t="inlineStr">
+        <is>
+          <t>BIBS Product Owner</t>
+        </is>
+      </c>
+      <c r="I115" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="J115" s="22" t="inlineStr">
+        <is>
+          <t>Issued for BDOI review</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="12" t="inlineStr">
+        <is>
+          <t>BRD-13</t>
+        </is>
+      </c>
+      <c r="B116" s="12" t="inlineStr">
+        <is>
+          <t>FitGap</t>
+        </is>
+      </c>
+      <c r="C116" s="12" t="inlineStr">
+        <is>
+          <t>Data Migration BRD vs OOTB vs Best Practice</t>
+        </is>
+      </c>
+      <c r="D116" s="12" t="inlineStr">
+        <is>
+          <t>BIBS_FitGap_BRD-13_Data_Migration_BRD_vs_OOTB_vs_Best_Practice_v1.0</t>
+        </is>
+      </c>
+      <c r="E116" s="12" t="inlineStr">
+        <is>
+          <t>XLSX</t>
+        </is>
+      </c>
+      <c r="F116" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G116" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H116" s="12" t="inlineStr">
+        <is>
+          <t>BIBS Product Owner</t>
+        </is>
+      </c>
+      <c r="I116" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="J116" s="22" t="inlineStr">
+        <is>
+          <t>Issued for BDOI review</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="12" t="inlineStr">
+        <is>
           <t>Programme</t>
         </is>
       </c>
-      <c r="B111" s="12" t="inlineStr">
+      <c r="B117" s="12" t="inlineStr">
         <is>
           <t>Conformance</t>
         </is>
       </c>
-      <c r="C111" s="12" t="inlineStr">
+      <c r="C117" s="12" t="inlineStr">
         <is>
           <t>End-to-End Conformance Register</t>
         </is>
       </c>
-      <c r="D111" s="12" t="inlineStr">
+      <c r="D117" s="12" t="inlineStr">
         <is>
           <t>BIBS_Conformance_BRD-00_End-to-End_Conformance_Register_v1.7</t>
         </is>
       </c>
-      <c r="E111" s="12" t="inlineStr">
+      <c r="E117" s="12" t="inlineStr">
         <is>
           <t>XLSX</t>
         </is>
       </c>
-      <c r="F111" s="12" t="inlineStr">
+      <c r="F117" s="12" t="inlineStr">
         <is>
           <t>1.7</t>
         </is>
       </c>
-      <c r="G111" s="12" t="inlineStr">
+      <c r="G117" s="12" t="inlineStr">
         <is>
           <t>17 Oct 2026</t>
         </is>
       </c>
-      <c r="H111" s="12" t="inlineStr">
+      <c r="H117" s="12" t="inlineStr">
         <is>
           <t>BIBS Product Owner</t>
         </is>
       </c>
-      <c r="I111" s="12" t="inlineStr">
-        <is>
-          <t>iorta TechNXT Project Team</t>
-        </is>
-      </c>
-      <c r="J111" s="22" t="inlineStr">
+      <c r="I117" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="J117" s="22" t="inlineStr">
         <is>
           <t>Issued for BDOI review</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J111"/>
+  <autoFilter ref="A4:J117"/>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:J611">
+  <conditionalFormatting sqref="A5:J617">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J5:J611" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
+    <dataValidation sqref="J5:J617" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
       <formula1>'Lists'!$A$2:$A$5</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>